<commit_message>
Update - Linkedin day-86
</commit_message>
<xml_diff>
--- a/LinkedIN-Posts.xlsx
+++ b/LinkedIN-Posts.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="88">
   <si>
     <t>Days</t>
   </si>
@@ -285,6 +285,9 @@
   </si>
   <si>
     <t>https://www.linkedin.com/posts/venkatesh-gangavarapu_devops-kubernetes-k8s-share-7486727367709605888-_8ls/</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/venkatesh-gangavarapu_devops-ansible-ssh-share-7487085870932525056-vyfl/</t>
   </si>
 </sst>
 </file>
@@ -1311,6 +1314,9 @@
       <c r="A87">
         <v>86</v>
       </c>
+      <c r="B87" s="1" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88">
@@ -1469,6 +1475,7 @@
     <hyperlink ref="B52" r:id="rId83"/>
     <hyperlink ref="B65" r:id="rId84"/>
     <hyperlink ref="B68" r:id="rId85"/>
+    <hyperlink ref="B87" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>